<commit_message>
Update test cases and Excel files for quiz core flow
- Modified TC_Login.xlsx and TC_QuizCoreFlow.xlsx files to reflect the latest test cases.
- Added temporary files for TC_Login and TC_QuizCoreFlow to track unsaved changes.
- Implemented comprehensive Selenium tests for the quiz core flow, covering various scenarios including quiz navigation, question answering, and result validation.
- Enhanced error handling and logging for better traceability during test execution.
</commit_message>
<xml_diff>
--- a/data/TC_Login.xlsx
+++ b/data/TC_Login.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Đồ án\quiz-trivia-tooltest\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D18908A-16EF-422C-AE6D-F9B03E57436F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C206107-D35E-4E6E-BF6A-7B832F220D58}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="34452" yWindow="1188" windowWidth="30936" windowHeight="16776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="347" uniqueCount="221">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="347" uniqueCount="223">
   <si>
     <t>Project</t>
   </si>
@@ -266,9 +266,6 @@
     <t>Email with leading/trailing spaces</t>
   </si>
   <si>
-    <t xml:space="preserve">  user@test.com  </t>
-  </si>
-  <si>
     <t>Login succeeds (email trimmed automatically)</t>
   </si>
   <si>
@@ -684,13 +681,22 @@
   </si>
   <si>
     <t>Firestore rule blocks read of non-public</t>
+  </si>
+  <si>
+    <t>nguyenvivi73@gmail.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  nguyenvivi73@gmail.com  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">nguyenvivi73@gmail.com </t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -726,14 +732,6 @@
       <sz val="10"/>
       <color rgb="FF9C0006"/>
       <name val="Arial"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color theme="10"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="8">
@@ -822,11 +820,10 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -845,16 +842,11 @@
     <xf numFmtId="0" fontId="5" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
   </cellXfs>
-  <cellStyles count="2">
-    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -1176,111 +1168,111 @@
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="10" t="s">
+      <c r="B1" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="11"/>
-      <c r="D1" s="11"/>
-      <c r="E1" s="11"/>
-      <c r="F1" s="11"/>
-      <c r="G1" s="11"/>
-      <c r="H1" s="11"/>
-      <c r="I1" s="11"/>
-      <c r="J1" s="11"/>
-      <c r="K1" s="11"/>
-      <c r="L1" s="11"/>
-      <c r="M1" s="12"/>
+      <c r="C1" s="9"/>
+      <c r="D1" s="9"/>
+      <c r="E1" s="9"/>
+      <c r="F1" s="9"/>
+      <c r="G1" s="9"/>
+      <c r="H1" s="9"/>
+      <c r="I1" s="9"/>
+      <c r="J1" s="9"/>
+      <c r="K1" s="9"/>
+      <c r="L1" s="9"/>
+      <c r="M1" s="10"/>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="10" t="s">
+      <c r="B2" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="C2" s="11"/>
-      <c r="D2" s="11"/>
-      <c r="E2" s="11"/>
-      <c r="F2" s="11"/>
-      <c r="G2" s="11"/>
-      <c r="H2" s="11"/>
-      <c r="I2" s="11"/>
-      <c r="J2" s="11"/>
-      <c r="K2" s="11"/>
-      <c r="L2" s="11"/>
-      <c r="M2" s="12"/>
+      <c r="C2" s="9"/>
+      <c r="D2" s="9"/>
+      <c r="E2" s="9"/>
+      <c r="F2" s="9"/>
+      <c r="G2" s="9"/>
+      <c r="H2" s="9"/>
+      <c r="I2" s="9"/>
+      <c r="J2" s="9"/>
+      <c r="K2" s="9"/>
+      <c r="L2" s="9"/>
+      <c r="M2" s="10"/>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A3" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="10" t="s">
+      <c r="B3" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="C3" s="11"/>
-      <c r="D3" s="11"/>
-      <c r="E3" s="11"/>
-      <c r="F3" s="11"/>
-      <c r="G3" s="11"/>
-      <c r="H3" s="11"/>
-      <c r="I3" s="11"/>
-      <c r="J3" s="11"/>
-      <c r="K3" s="11"/>
-      <c r="L3" s="11"/>
-      <c r="M3" s="12"/>
+      <c r="C3" s="9"/>
+      <c r="D3" s="9"/>
+      <c r="E3" s="9"/>
+      <c r="F3" s="9"/>
+      <c r="G3" s="9"/>
+      <c r="H3" s="9"/>
+      <c r="I3" s="9"/>
+      <c r="J3" s="9"/>
+      <c r="K3" s="9"/>
+      <c r="L3" s="9"/>
+      <c r="M3" s="10"/>
     </row>
     <row r="4" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A4" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="10" t="s">
+      <c r="B4" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="C4" s="11"/>
-      <c r="D4" s="11"/>
-      <c r="E4" s="11"/>
-      <c r="F4" s="11"/>
-      <c r="G4" s="11"/>
-      <c r="H4" s="11"/>
-      <c r="I4" s="11"/>
-      <c r="J4" s="11"/>
-      <c r="K4" s="11"/>
-      <c r="L4" s="11"/>
-      <c r="M4" s="12"/>
+      <c r="C4" s="9"/>
+      <c r="D4" s="9"/>
+      <c r="E4" s="9"/>
+      <c r="F4" s="9"/>
+      <c r="G4" s="9"/>
+      <c r="H4" s="9"/>
+      <c r="I4" s="9"/>
+      <c r="J4" s="9"/>
+      <c r="K4" s="9"/>
+      <c r="L4" s="9"/>
+      <c r="M4" s="10"/>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A5" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="10"/>
-      <c r="C5" s="11"/>
-      <c r="D5" s="11"/>
-      <c r="E5" s="11"/>
-      <c r="F5" s="11"/>
-      <c r="G5" s="11"/>
-      <c r="H5" s="11"/>
-      <c r="I5" s="11"/>
-      <c r="J5" s="11"/>
-      <c r="K5" s="11"/>
-      <c r="L5" s="11"/>
-      <c r="M5" s="12"/>
+      <c r="B5" s="8"/>
+      <c r="C5" s="9"/>
+      <c r="D5" s="9"/>
+      <c r="E5" s="9"/>
+      <c r="F5" s="9"/>
+      <c r="G5" s="9"/>
+      <c r="H5" s="9"/>
+      <c r="I5" s="9"/>
+      <c r="J5" s="9"/>
+      <c r="K5" s="9"/>
+      <c r="L5" s="9"/>
+      <c r="M5" s="10"/>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A6" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B6" s="10"/>
-      <c r="C6" s="11"/>
-      <c r="D6" s="11"/>
-      <c r="E6" s="11"/>
-      <c r="F6" s="11"/>
-      <c r="G6" s="11"/>
-      <c r="H6" s="11"/>
-      <c r="I6" s="11"/>
-      <c r="J6" s="11"/>
-      <c r="K6" s="11"/>
-      <c r="L6" s="11"/>
-      <c r="M6" s="12"/>
+      <c r="B6" s="8"/>
+      <c r="C6" s="9"/>
+      <c r="D6" s="9"/>
+      <c r="E6" s="9"/>
+      <c r="F6" s="9"/>
+      <c r="G6" s="9"/>
+      <c r="H6" s="9"/>
+      <c r="I6" s="9"/>
+      <c r="J6" s="9"/>
+      <c r="K6" s="9"/>
+      <c r="L6" s="9"/>
+      <c r="M6" s="10"/>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A7" s="3" t="s">
@@ -1336,7 +1328,7 @@
       <c r="D8" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="E8" s="8" t="s">
+      <c r="E8" t="s">
         <v>27</v>
       </c>
       <c r="F8" s="4" t="s">
@@ -1377,7 +1369,7 @@
       <c r="D9" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="E9" s="8" t="s">
+      <c r="E9" s="6" t="s">
         <v>27</v>
       </c>
       <c r="F9" s="6" t="s">
@@ -1418,7 +1410,7 @@
       <c r="D10" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="E10" s="9" t="s">
+      <c r="E10" t="s">
         <v>48</v>
       </c>
       <c r="F10" s="4" t="s">
@@ -1498,10 +1490,9 @@
       <c r="D12" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="E12" s="4" t="s">
-        <v>64</v>
-      </c>
-      <c r="F12" s="4"/>
+      <c r="E12" t="s">
+        <v>220</v>
+      </c>
       <c r="G12" s="4" t="s">
         <v>65</v>
       </c>
@@ -1578,13 +1569,13 @@
       <c r="D14" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="E14" s="4" t="s">
-        <v>64</v>
+      <c r="E14" t="s">
+        <v>220</v>
       </c>
       <c r="F14" s="4" t="s">
         <v>75</v>
       </c>
-      <c r="G14" s="4" t="s">
+      <c r="G14" t="s">
         <v>76</v>
       </c>
       <c r="H14" s="4" t="s">
@@ -1620,54 +1611,54 @@
         <v>56</v>
       </c>
       <c r="E15" s="6" t="s">
-        <v>81</v>
+        <v>221</v>
       </c>
       <c r="F15" s="6" t="s">
         <v>57</v>
       </c>
       <c r="G15" s="6" t="s">
+        <v>81</v>
+      </c>
+      <c r="H15" s="6" t="s">
         <v>82</v>
       </c>
-      <c r="H15" s="6" t="s">
+      <c r="I15" s="6" t="s">
         <v>83</v>
       </c>
-      <c r="I15" s="6" t="s">
+      <c r="J15" s="6" t="s">
         <v>84</v>
       </c>
-      <c r="J15" s="6" t="s">
+      <c r="K15" s="6" t="s">
         <v>85</v>
-      </c>
-      <c r="K15" s="6" t="s">
-        <v>86</v>
       </c>
       <c r="L15" s="5" t="s">
         <v>34</v>
       </c>
       <c r="M15" s="6" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="16" spans="1:13" ht="127.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A16" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="B16" s="4" t="s">
         <v>88</v>
       </c>
-      <c r="B16" s="4" t="s">
+      <c r="C16" s="4" t="s">
         <v>89</v>
       </c>
-      <c r="C16" s="4" t="s">
+      <c r="D16" s="4" t="s">
         <v>90</v>
       </c>
-      <c r="D16" s="4" t="s">
+      <c r="E16" s="4" t="s">
         <v>91</v>
-      </c>
-      <c r="E16" s="4" t="s">
-        <v>92</v>
       </c>
       <c r="F16" s="4" t="s">
         <v>57</v>
       </c>
       <c r="G16" s="4" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="H16" s="4" t="s">
         <v>77</v>
@@ -1678,69 +1669,69 @@
       <c r="J16" s="4"/>
       <c r="K16" s="4"/>
       <c r="L16" s="5" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="M16" s="4"/>
     </row>
     <row r="17" spans="1:13" ht="25.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A17" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="B17" s="6" t="s">
         <v>95</v>
       </c>
-      <c r="B17" s="6" t="s">
+      <c r="C17" s="6" t="s">
         <v>96</v>
       </c>
-      <c r="C17" s="6" t="s">
+      <c r="D17" s="6" t="s">
         <v>97</v>
       </c>
-      <c r="D17" s="6" t="s">
-        <v>98</v>
-      </c>
       <c r="E17" s="6" t="s">
-        <v>64</v>
+        <v>222</v>
       </c>
       <c r="F17" s="6" t="s">
         <v>57</v>
       </c>
       <c r="G17" s="6" t="s">
+        <v>98</v>
+      </c>
+      <c r="H17" s="6" t="s">
         <v>99</v>
       </c>
-      <c r="H17" s="6" t="s">
-        <v>100</v>
-      </c>
       <c r="I17" s="6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="J17" s="6"/>
       <c r="K17" s="6"/>
       <c r="L17" s="5" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="M17" s="6"/>
     </row>
     <row r="18" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A18" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="B18" s="4" t="s">
         <v>101</v>
-      </c>
-      <c r="B18" s="4" t="s">
-        <v>102</v>
       </c>
       <c r="C18" s="4" t="s">
         <v>38</v>
       </c>
       <c r="D18" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="E18" s="4" t="s">
         <v>103</v>
-      </c>
-      <c r="E18" s="4" t="s">
-        <v>104</v>
       </c>
       <c r="F18" s="4" t="s">
         <v>57</v>
       </c>
       <c r="G18" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="H18" s="4" t="s">
         <v>105</v>
-      </c>
-      <c r="H18" s="4" t="s">
-        <v>106</v>
       </c>
       <c r="I18" s="4" t="s">
         <v>51</v>
@@ -1748,31 +1739,31 @@
       <c r="J18" s="4"/>
       <c r="K18" s="4"/>
       <c r="L18" s="5" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="M18" s="4"/>
     </row>
     <row r="19" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A19" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B19" s="6" t="s">
         <v>107</v>
-      </c>
-      <c r="B19" s="6" t="s">
-        <v>108</v>
       </c>
       <c r="C19" s="6" t="s">
         <v>38</v>
       </c>
       <c r="D19" s="6" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="E19" s="6" t="s">
         <v>64</v>
       </c>
       <c r="F19" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="G19" s="6" t="s">
         <v>109</v>
-      </c>
-      <c r="G19" s="6" t="s">
-        <v>110</v>
       </c>
       <c r="H19" s="6" t="s">
         <v>77</v>
@@ -1783,16 +1774,16 @@
       <c r="J19" s="6"/>
       <c r="K19" s="6"/>
       <c r="L19" s="5" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="M19" s="6"/>
     </row>
     <row r="20" spans="1:13" ht="25.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A20" s="4" t="s">
+        <v>110</v>
+      </c>
+      <c r="B20" s="4" t="s">
         <v>111</v>
-      </c>
-      <c r="B20" s="4" t="s">
-        <v>112</v>
       </c>
       <c r="C20" s="4" t="s">
         <v>25</v>
@@ -1801,16 +1792,16 @@
         <v>26</v>
       </c>
       <c r="E20" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="F20" s="4" t="s">
         <v>113</v>
       </c>
-      <c r="F20" s="4" t="s">
+      <c r="G20" s="4" t="s">
         <v>114</v>
       </c>
-      <c r="G20" s="4" t="s">
+      <c r="H20" s="4" t="s">
         <v>115</v>
-      </c>
-      <c r="H20" s="4" t="s">
-        <v>116</v>
       </c>
       <c r="I20" s="4" t="s">
         <v>31</v>
@@ -1818,33 +1809,33 @@
       <c r="J20" s="4"/>
       <c r="K20" s="4"/>
       <c r="L20" s="5" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="M20" s="4" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="21" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A21" s="6" t="s">
+        <v>117</v>
+      </c>
+      <c r="B21" s="6" t="s">
         <v>118</v>
       </c>
-      <c r="B21" s="6" t="s">
+      <c r="C21" s="6" t="s">
         <v>119</v>
       </c>
-      <c r="C21" s="6" t="s">
+      <c r="D21" s="6" t="s">
+        <v>102</v>
+      </c>
+      <c r="E21" s="6" t="s">
         <v>120</v>
       </c>
-      <c r="D21" s="6" t="s">
-        <v>103</v>
-      </c>
-      <c r="E21" s="6" t="s">
+      <c r="F21" s="6" t="s">
         <v>121</v>
       </c>
-      <c r="F21" s="6" t="s">
+      <c r="G21" s="6" t="s">
         <v>122</v>
-      </c>
-      <c r="G21" s="6" t="s">
-        <v>123</v>
       </c>
       <c r="H21" s="6" t="s">
         <v>77</v>
@@ -1855,21 +1846,21 @@
       <c r="J21" s="6"/>
       <c r="K21" s="6"/>
       <c r="L21" s="5" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="M21" s="6" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="22" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A22" s="4" t="s">
+        <v>124</v>
+      </c>
+      <c r="B22" s="4" t="s">
         <v>125</v>
       </c>
-      <c r="B22" s="4" t="s">
+      <c r="C22" s="4" t="s">
         <v>126</v>
-      </c>
-      <c r="C22" s="4" t="s">
-        <v>127</v>
       </c>
       <c r="D22" s="4" t="s">
         <v>26</v>
@@ -1881,33 +1872,33 @@
         <v>57</v>
       </c>
       <c r="G22" s="4" t="s">
+        <v>127</v>
+      </c>
+      <c r="H22" s="4" t="s">
         <v>128</v>
       </c>
-      <c r="H22" s="4" t="s">
+      <c r="I22" s="4" t="s">
         <v>129</v>
-      </c>
-      <c r="I22" s="4" t="s">
-        <v>130</v>
       </c>
       <c r="J22" s="4"/>
       <c r="K22" s="4"/>
       <c r="L22" s="5" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="M22" s="4"/>
     </row>
     <row r="23" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A23" s="6" t="s">
+        <v>130</v>
+      </c>
+      <c r="B23" s="6" t="s">
         <v>131</v>
       </c>
-      <c r="B23" s="6" t="s">
-        <v>132</v>
-      </c>
       <c r="C23" s="6" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="D23" s="6" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="E23" s="6" t="s">
         <v>64</v>
@@ -1916,33 +1907,33 @@
         <v>57</v>
       </c>
       <c r="G23" s="6" t="s">
+        <v>132</v>
+      </c>
+      <c r="H23" s="6" t="s">
         <v>133</v>
       </c>
-      <c r="H23" s="6" t="s">
+      <c r="I23" s="6" t="s">
         <v>134</v>
-      </c>
-      <c r="I23" s="6" t="s">
-        <v>135</v>
       </c>
       <c r="J23" s="6"/>
       <c r="K23" s="6"/>
       <c r="L23" s="5" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="M23" s="6"/>
     </row>
     <row r="24" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A24" s="4" t="s">
+        <v>135</v>
+      </c>
+      <c r="B24" s="4" t="s">
         <v>136</v>
       </c>
-      <c r="B24" s="4" t="s">
+      <c r="C24" s="4" t="s">
         <v>137</v>
       </c>
-      <c r="C24" s="4" t="s">
+      <c r="D24" s="4" t="s">
         <v>138</v>
-      </c>
-      <c r="D24" s="4" t="s">
-        <v>139</v>
       </c>
       <c r="E24" s="4" t="s">
         <v>64</v>
@@ -1951,27 +1942,27 @@
         <v>57</v>
       </c>
       <c r="G24" s="4" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="H24" s="4" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="I24" s="4" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="J24" s="4"/>
       <c r="K24" s="4"/>
       <c r="L24" s="5" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="M24" s="4"/>
     </row>
     <row r="25" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A25" s="6" t="s">
+        <v>140</v>
+      </c>
+      <c r="B25" s="6" t="s">
         <v>141</v>
-      </c>
-      <c r="B25" s="6" t="s">
-        <v>142</v>
       </c>
       <c r="C25" s="6" t="s">
         <v>25</v>
@@ -1983,13 +1974,13 @@
         <v>64</v>
       </c>
       <c r="F25" s="6" t="s">
+        <v>142</v>
+      </c>
+      <c r="G25" s="6" t="s">
         <v>143</v>
       </c>
-      <c r="G25" s="6" t="s">
+      <c r="H25" s="6" t="s">
         <v>144</v>
-      </c>
-      <c r="H25" s="6" t="s">
-        <v>145</v>
       </c>
       <c r="I25" s="6" t="s">
         <v>51</v>
@@ -1997,18 +1988,18 @@
       <c r="J25" s="6"/>
       <c r="K25" s="6"/>
       <c r="L25" s="7" t="s">
+        <v>145</v>
+      </c>
+      <c r="M25" s="6" t="s">
         <v>146</v>
-      </c>
-      <c r="M25" s="6" t="s">
-        <v>147</v>
       </c>
     </row>
     <row r="26" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A26" s="4" t="s">
+        <v>147</v>
+      </c>
+      <c r="B26" s="4" t="s">
         <v>148</v>
-      </c>
-      <c r="B26" s="4" t="s">
-        <v>149</v>
       </c>
       <c r="C26" s="4" t="s">
         <v>38</v>
@@ -2017,16 +2008,16 @@
         <v>26</v>
       </c>
       <c r="E26" s="4" t="s">
+        <v>149</v>
+      </c>
+      <c r="F26" s="4" t="s">
+        <v>121</v>
+      </c>
+      <c r="G26" s="4" t="s">
         <v>150</v>
       </c>
-      <c r="F26" s="4" t="s">
-        <v>122</v>
-      </c>
-      <c r="G26" s="4" t="s">
+      <c r="H26" s="4" t="s">
         <v>151</v>
-      </c>
-      <c r="H26" s="4" t="s">
-        <v>152</v>
       </c>
       <c r="I26" s="4" t="s">
         <v>51</v>
@@ -2034,18 +2025,18 @@
       <c r="J26" s="4"/>
       <c r="K26" s="4"/>
       <c r="L26" s="7" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="M26" s="4" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="27" spans="1:13" ht="25.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A27" s="6" t="s">
+        <v>153</v>
+      </c>
+      <c r="B27" s="6" t="s">
         <v>154</v>
-      </c>
-      <c r="B27" s="6" t="s">
-        <v>155</v>
       </c>
       <c r="C27" s="6" t="s">
         <v>25</v>
@@ -2054,27 +2045,27 @@
         <v>26</v>
       </c>
       <c r="E27" s="6" t="s">
+        <v>155</v>
+      </c>
+      <c r="F27" s="6" t="s">
         <v>156</v>
       </c>
-      <c r="F27" s="6" t="s">
+      <c r="G27" s="6" t="s">
         <v>157</v>
       </c>
-      <c r="G27" s="6" t="s">
+      <c r="H27" s="6" t="s">
         <v>158</v>
       </c>
-      <c r="H27" s="6" t="s">
+      <c r="I27" s="6" t="s">
         <v>159</v>
-      </c>
-      <c r="I27" s="6" t="s">
-        <v>160</v>
       </c>
       <c r="J27" s="6"/>
       <c r="K27" s="6"/>
       <c r="L27" s="7" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="M27" s="6" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
     </row>
   </sheetData>
@@ -2088,8 +2079,8 @@
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="E8" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
-    <hyperlink ref="E9" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
-    <hyperlink ref="E10" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
+    <hyperlink ref="E10" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
+    <hyperlink ref="E14" r:id="rId3" xr:uid="{36C41BC0-033E-4BAD-8582-4CC29949F8E8}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2124,7 +2115,7 @@
         <v>2</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.45">
@@ -2140,7 +2131,7 @@
         <v>6</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.45">
@@ -2151,19 +2142,19 @@
         <v>11</v>
       </c>
       <c r="C5" s="3" t="s">
+        <v>163</v>
+      </c>
+      <c r="D5" s="3" t="s">
         <v>164</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="E5" s="3" t="s">
         <v>165</v>
       </c>
-      <c r="E5" s="3" t="s">
+      <c r="F5" s="3" t="s">
         <v>166</v>
       </c>
-      <c r="F5" s="3" t="s">
+      <c r="G5" s="3" t="s">
         <v>167</v>
-      </c>
-      <c r="G5" s="3" t="s">
-        <v>168</v>
       </c>
       <c r="H5" s="3" t="s">
         <v>21</v>
@@ -2174,271 +2165,271 @@
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A6" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="B6" s="4" t="s">
         <v>169</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="C6" s="4" t="s">
         <v>170</v>
       </c>
-      <c r="C6" s="4" t="s">
+      <c r="D6" s="4" t="s">
         <v>171</v>
       </c>
-      <c r="D6" s="4" t="s">
+      <c r="E6" s="4" t="s">
         <v>172</v>
       </c>
-      <c r="E6" s="4" t="s">
+      <c r="F6" s="4" t="s">
         <v>173</v>
       </c>
-      <c r="F6" s="4" t="s">
-        <v>174</v>
-      </c>
       <c r="G6" s="4" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="H6" s="5" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="I6" s="4"/>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A7" s="6" t="s">
+        <v>174</v>
+      </c>
+      <c r="B7" s="6" t="s">
         <v>175</v>
       </c>
-      <c r="B7" s="6" t="s">
+      <c r="C7" s="6" t="s">
+        <v>170</v>
+      </c>
+      <c r="D7" s="6" t="s">
         <v>176</v>
       </c>
-      <c r="C7" s="6" t="s">
-        <v>171</v>
-      </c>
-      <c r="D7" s="6" t="s">
+      <c r="E7" s="6" t="s">
         <v>177</v>
       </c>
-      <c r="E7" s="6" t="s">
+      <c r="F7" s="6" t="s">
         <v>178</v>
       </c>
-      <c r="F7" s="6" t="s">
-        <v>179</v>
-      </c>
       <c r="G7" s="6" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="H7" s="5" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="I7" s="6"/>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A8" s="4" t="s">
+        <v>179</v>
+      </c>
+      <c r="B8" s="4" t="s">
         <v>180</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="C8" s="4" t="s">
+        <v>170</v>
+      </c>
+      <c r="D8" s="4" t="s">
         <v>181</v>
       </c>
-      <c r="C8" s="4" t="s">
-        <v>171</v>
-      </c>
-      <c r="D8" s="4" t="s">
+      <c r="E8" s="4" t="s">
         <v>182</v>
       </c>
-      <c r="E8" s="4" t="s">
+      <c r="F8" s="4" t="s">
         <v>183</v>
       </c>
-      <c r="F8" s="4" t="s">
-        <v>184</v>
-      </c>
       <c r="G8" s="4" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="H8" s="5" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="I8" s="4"/>
     </row>
     <row r="9" spans="1:9" ht="25.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A9" s="6" t="s">
+        <v>184</v>
+      </c>
+      <c r="B9" s="6" t="s">
         <v>185</v>
       </c>
-      <c r="B9" s="6" t="s">
+      <c r="C9" s="6" t="s">
         <v>186</v>
       </c>
-      <c r="C9" s="6" t="s">
+      <c r="D9" s="6" t="s">
         <v>187</v>
       </c>
-      <c r="D9" s="6" t="s">
+      <c r="E9" s="6" t="s">
         <v>188</v>
       </c>
-      <c r="E9" s="6" t="s">
+      <c r="F9" s="6" t="s">
         <v>189</v>
       </c>
-      <c r="F9" s="6" t="s">
-        <v>190</v>
-      </c>
       <c r="G9" s="6" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="H9" s="5" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="I9" s="6"/>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A10" s="4" t="s">
+        <v>190</v>
+      </c>
+      <c r="B10" s="4" t="s">
         <v>191</v>
       </c>
-      <c r="B10" s="4" t="s">
+      <c r="C10" s="4" t="s">
+        <v>186</v>
+      </c>
+      <c r="D10" s="4" t="s">
         <v>192</v>
       </c>
-      <c r="C10" s="4" t="s">
-        <v>187</v>
-      </c>
-      <c r="D10" s="4" t="s">
+      <c r="E10" s="4" t="s">
         <v>193</v>
       </c>
-      <c r="E10" s="4" t="s">
+      <c r="F10" s="4" t="s">
         <v>194</v>
       </c>
-      <c r="F10" s="4" t="s">
-        <v>195</v>
-      </c>
       <c r="G10" s="4" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="H10" s="5" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="I10" s="4"/>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A11" s="6" t="s">
+        <v>195</v>
+      </c>
+      <c r="B11" s="6" t="s">
         <v>196</v>
       </c>
-      <c r="B11" s="6" t="s">
+      <c r="C11" s="6" t="s">
         <v>197</v>
       </c>
-      <c r="C11" s="6" t="s">
+      <c r="D11" s="6" t="s">
+        <v>192</v>
+      </c>
+      <c r="E11" s="6" t="s">
         <v>198</v>
       </c>
-      <c r="D11" s="6" t="s">
-        <v>193</v>
-      </c>
-      <c r="E11" s="6" t="s">
+      <c r="F11" s="6" t="s">
         <v>199</v>
       </c>
-      <c r="F11" s="6" t="s">
-        <v>200</v>
-      </c>
       <c r="G11" s="6" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="H11" s="5" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="I11" s="6"/>
     </row>
     <row r="12" spans="1:9" ht="25.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A12" s="4" t="s">
+        <v>200</v>
+      </c>
+      <c r="B12" s="4" t="s">
         <v>201</v>
       </c>
-      <c r="B12" s="4" t="s">
+      <c r="C12" s="4" t="s">
+        <v>170</v>
+      </c>
+      <c r="D12" s="4" t="s">
         <v>202</v>
       </c>
-      <c r="C12" s="4" t="s">
-        <v>171</v>
-      </c>
-      <c r="D12" s="4" t="s">
+      <c r="E12" s="4" t="s">
         <v>203</v>
       </c>
-      <c r="E12" s="4" t="s">
+      <c r="F12" s="4" t="s">
         <v>204</v>
       </c>
-      <c r="F12" s="4" t="s">
-        <v>205</v>
-      </c>
       <c r="G12" s="4" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="H12" s="5" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="I12" s="4"/>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A13" s="6" t="s">
+        <v>205</v>
+      </c>
+      <c r="B13" s="6" t="s">
         <v>206</v>
       </c>
-      <c r="B13" s="6" t="s">
+      <c r="C13" s="6" t="s">
+        <v>170</v>
+      </c>
+      <c r="D13" s="6" t="s">
         <v>207</v>
       </c>
-      <c r="C13" s="6" t="s">
-        <v>171</v>
-      </c>
-      <c r="D13" s="6" t="s">
+      <c r="E13" s="6" t="s">
         <v>208</v>
       </c>
-      <c r="E13" s="6" t="s">
+      <c r="F13" s="6" t="s">
         <v>209</v>
       </c>
-      <c r="F13" s="6" t="s">
-        <v>210</v>
-      </c>
       <c r="G13" s="6" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="H13" s="5" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="I13" s="6"/>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A14" s="4" t="s">
+        <v>210</v>
+      </c>
+      <c r="B14" s="4" t="s">
         <v>211</v>
       </c>
-      <c r="B14" s="4" t="s">
+      <c r="C14" s="4" t="s">
+        <v>186</v>
+      </c>
+      <c r="D14" s="4" t="s">
         <v>212</v>
       </c>
-      <c r="C14" s="4" t="s">
-        <v>187</v>
-      </c>
-      <c r="D14" s="4" t="s">
+      <c r="E14" s="4" t="s">
         <v>213</v>
       </c>
-      <c r="E14" s="4" t="s">
+      <c r="F14" s="4" t="s">
         <v>214</v>
       </c>
-      <c r="F14" s="4" t="s">
-        <v>215</v>
-      </c>
       <c r="G14" s="4" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="H14" s="5" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="I14" s="4"/>
     </row>
     <row r="15" spans="1:9" ht="25.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A15" s="6" t="s">
+        <v>215</v>
+      </c>
+      <c r="B15" s="6" t="s">
         <v>216</v>
       </c>
-      <c r="B15" s="6" t="s">
+      <c r="C15" s="6" t="s">
+        <v>170</v>
+      </c>
+      <c r="D15" s="6" t="s">
         <v>217</v>
       </c>
-      <c r="C15" s="6" t="s">
-        <v>171</v>
-      </c>
-      <c r="D15" s="6" t="s">
+      <c r="E15" s="6" t="s">
         <v>218</v>
       </c>
-      <c r="E15" s="6" t="s">
+      <c r="F15" s="6" t="s">
         <v>219</v>
       </c>
-      <c r="F15" s="6" t="s">
-        <v>220</v>
-      </c>
       <c r="G15" s="6" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="H15" s="5" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="I15" s="6"/>
     </row>

</xml_diff>

<commit_message>
feat: add login test case data spreadsheet
</commit_message>
<xml_diff>
--- a/data/TC_Login.xlsx
+++ b/data/TC_Login.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Đồ án\quiz-trivia-tooltest\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C206107-D35E-4E6E-BF6A-7B832F220D58}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{75D4A7CB-7469-4128-8DAD-A83211579780}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="34452" yWindow="1188" windowWidth="30936" windowHeight="16776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="347" uniqueCount="223">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="372" uniqueCount="241">
   <si>
     <t>Project</t>
   </si>
@@ -215,336 +215,420 @@
     <t>Empty password field</t>
   </si>
   <si>
+    <t>nguyenvivi73@gmail.com</t>
+  </si>
+  <si>
+    <t>Inline error: 'Mật khẩu là bắt buộc'</t>
+  </si>
+  <si>
+    <t>Toast: 'Mật khẩu là bắt buộc'; URL: https://datn-quizapp.web.app/login</t>
+  </si>
+  <si>
+    <t>TC-RBAC-VAL-03</t>
+  </si>
+  <si>
+    <t>Invalid email format</t>
+  </si>
+  <si>
+    <t>not-an-email</t>
+  </si>
+  <si>
+    <t>Inline error: email format invalid</t>
+  </si>
+  <si>
+    <t>Toast: 'Email không hợp lệ'; URL: https://datn-quizapp.web.app/login</t>
+  </si>
+  <si>
+    <t>No auth call made (invalid email format rejected client-side)</t>
+  </si>
+  <si>
+    <t>TC-RBAC-VAL-04</t>
+  </si>
+  <si>
+    <t>Whitespace-only password</t>
+  </si>
+  <si>
+    <t xml:space="preserve">     </t>
+  </si>
+  <si>
+    <t>Error: incorrect email or password</t>
+  </si>
+  <si>
+    <t>No session created</t>
+  </si>
+  <si>
+    <t>No session created (whitespace password rejected)</t>
+  </si>
+  <si>
+    <t>TC-RBAC-VAL-05</t>
+  </si>
+  <si>
+    <t>Email with leading/trailing spaces</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  nguyenvivi73@gmail.com  </t>
+  </si>
+  <si>
+    <t>Login succeeds (email trimmed automatically)</t>
+  </si>
+  <si>
+    <t>Session created normally</t>
+  </si>
+  <si>
+    <t>Sign out</t>
+  </si>
+  <si>
+    <t>Redirected away from /login: True; URL: https://datn-quizapp.web.app/dashboard</t>
+  </si>
+  <si>
+    <t>Session created for nguyenvivi73@gmail.com</t>
+  </si>
+  <si>
+    <t>Trimming behavior | Run: 2026-04-18 11:30 | Run: 2026-04-18 11:49 | Run: 2026-04-18 11:51</t>
+  </si>
+  <si>
+    <t>TC-RBAC-VAL-06</t>
+  </si>
+  <si>
+    <t>Overlong email (&gt;256 chars)</t>
+  </si>
+  <si>
+    <t>BVA/Negative</t>
+  </si>
+  <si>
+    <t>Boundary</t>
+  </si>
+  <si>
+    <t>aaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaa@x.co</t>
+  </si>
+  <si>
+    <t>System stays stable; validation error shown</t>
+  </si>
+  <si>
+    <t>Toast: 'Email hoặc mật khẩu không đúng'; URL: https://datn-quizapp.web.app/login; System stable: True</t>
+  </si>
+  <si>
+    <t>No session created (overlong email rejected)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> | Run: 2026-04-22 07:31</t>
+  </si>
+  <si>
+    <t>TC-RBAC-NEG-01</t>
+  </si>
+  <si>
+    <t>Rapid repeated login clicks</t>
+  </si>
+  <si>
+    <t>Error Guessing</t>
+  </si>
+  <si>
+    <t>Negative</t>
+  </si>
+  <si>
+    <t xml:space="preserve">nguyenvivi73@gmail.com </t>
+  </si>
+  <si>
+    <t>Single login action processed; no duplicate sessions</t>
+  </si>
+  <si>
+    <t>Only 1 auth token created</t>
+  </si>
+  <si>
+    <t>Redirected after rapid clicks: False; URL: https://datn-quizapp.web.app/login</t>
+  </si>
+  <si>
+    <t>Could not verify via REST</t>
+  </si>
+  <si>
+    <t>TC-RBAC-NEG-02</t>
+  </si>
+  <si>
+    <t>XSS payload in email field</t>
+  </si>
+  <si>
+    <t>Security</t>
+  </si>
+  <si>
+    <t>&lt;script&gt;alert('xss')&lt;/script&gt;</t>
+  </si>
+  <si>
+    <t>Input rejected; no script executed</t>
+  </si>
+  <si>
+    <t>No auth attempt or error logged</t>
+  </si>
+  <si>
+    <t>XSS executed: False; Toast: 'Email không hợp lệ'; URL: https://datn-quizapp.web.app/login</t>
+  </si>
+  <si>
+    <t>No auth attempt with XSS payload (format rejected by Firebase)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> | Run: 2026-04-22 07:32</t>
+  </si>
+  <si>
+    <t>TC-RBAC-NEG-02b</t>
+  </si>
+  <si>
+    <t>SQL injection in password</t>
+  </si>
+  <si>
     <t>user@test.com</t>
   </si>
   <si>
-    <t>Inline error: 'Mật khẩu là bắt buộc'</t>
-  </si>
-  <si>
-    <t>Toast: 'Mật khẩu là bắt buộc'; URL: https://datn-quizapp.web.app/login</t>
-  </si>
-  <si>
-    <t>TC-RBAC-VAL-03</t>
-  </si>
-  <si>
-    <t>Invalid email format</t>
-  </si>
-  <si>
-    <t>not-an-email</t>
-  </si>
-  <si>
-    <t>Inline error: email format invalid</t>
-  </si>
-  <si>
-    <t>Toast: 'Email không hợp lệ'; URL: https://datn-quizapp.web.app/login</t>
-  </si>
-  <si>
-    <t>No auth call made (invalid email format rejected client-side)</t>
-  </si>
-  <si>
-    <t>TC-RBAC-VAL-04</t>
-  </si>
-  <si>
-    <t>Whitespace-only password</t>
-  </si>
-  <si>
-    <t xml:space="preserve">     </t>
-  </si>
-  <si>
-    <t>Error: incorrect email or password</t>
-  </si>
-  <si>
-    <t>No session created</t>
-  </si>
-  <si>
-    <t>No session created (whitespace password rejected)</t>
-  </si>
-  <si>
-    <t>TC-RBAC-VAL-05</t>
-  </si>
-  <si>
-    <t>Email with leading/trailing spaces</t>
-  </si>
-  <si>
-    <t>Login succeeds (email trimmed automatically)</t>
-  </si>
-  <si>
-    <t>Session created normally</t>
-  </si>
-  <si>
-    <t>Sign out</t>
-  </si>
-  <si>
-    <t>Redirected away from /login: True; URL: https://datn-quizapp.web.app/dashboard</t>
-  </si>
-  <si>
-    <t>Session created for nguyenvivi73@gmail.com</t>
-  </si>
-  <si>
-    <t>Trimming behavior | Run: 2026-04-18 11:30 | Run: 2026-04-18 11:49 | Run: 2026-04-18 11:51</t>
-  </si>
-  <si>
-    <t>TC-RBAC-VAL-06</t>
-  </si>
-  <si>
-    <t>Overlong email (&gt;256 chars)</t>
-  </si>
-  <si>
-    <t>BVA/Negative</t>
-  </si>
-  <si>
-    <t>Boundary</t>
-  </si>
-  <si>
-    <t>aaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaa@x.co</t>
-  </si>
-  <si>
-    <t>System stays stable; validation error shown</t>
+    <t>' OR '1'='1; --</t>
+  </si>
+  <si>
+    <t>Login fails; no data exposure</t>
+  </si>
+  <si>
+    <t>Firebase Auth is not SQL-backed; injection attempt harmless; Confirmed: no token issued</t>
+  </si>
+  <si>
+    <t>TC-RBAC-AUTH-08</t>
+  </si>
+  <si>
+    <t>Google OAuth login</t>
+  </si>
+  <si>
+    <t>(Google account)</t>
+  </si>
+  <si>
+    <t>(OAuth flow)</t>
+  </si>
+  <si>
+    <t>Redirect to dashboard; profile synced</t>
+  </si>
+  <si>
+    <t>Firestore users/{uid} created with role='user'</t>
+  </si>
+  <si>
+    <t>Google OAuth requires interactive account selection; skipped in headless Chrome</t>
+  </si>
+  <si>
+    <t>N/A – manual step required</t>
+  </si>
+  <si>
+    <t>SKIP</t>
+  </si>
+  <si>
+    <t>Manual step: select Google account | Run: 2026-04-22 07:32</t>
+  </si>
+  <si>
+    <t>TC-RBAC-ROLE-01</t>
+  </si>
+  <si>
+    <t>Guest access to protected route</t>
+  </si>
+  <si>
+    <t>Decision Table</t>
+  </si>
+  <si>
+    <t>(not logged in)</t>
+  </si>
+  <si>
+    <t>(none)</t>
+  </si>
+  <si>
+    <t>Redirect to /login page</t>
+  </si>
+  <si>
+    <t>Accessing /profile while logged out → URL: https://datn-quizapp.web.app/login</t>
+  </si>
+  <si>
+    <t>No session created (guest cannot create server-side state)</t>
+  </si>
+  <si>
+    <t>Navigate to /profile while logged out | Run: 2026-04-22 07:32</t>
+  </si>
+  <si>
+    <t>TC-RBAC-SES-03</t>
+  </si>
+  <si>
+    <t>Logout invalidates session</t>
+  </si>
+  <si>
+    <t>State Transition</t>
+  </si>
+  <si>
+    <t>Redirect to /login; protected pages blocked</t>
+  </si>
+  <si>
+    <t>Firebase ID token invalidated</t>
+  </si>
+  <si>
+    <t>N/A (logout is the action)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Logout UI interaction failed: Message: 
+Stacktrace:
+	chromedriver!GetHandleVerifier [0x7ff7941d0245+146d5]
+	chromedriver!GetHandleVerifier [0x7ff7941d02b0+14740]
+	chromedriver!(No symbol) [0x7ff793f3d7cd]
+	chromedriver!(No symbol) [0x7ff793f96c4e]
+	chromedriver!(No symbol) [0x7ff793f96f5c]
+	chromedriver!(No symbol) [0x7ff793fe7cc7]
+	chromedriver!(No symbol) [0x7ff793fe4818]
+	chromedriver!(No symbol) [0x7ff793f89018]
+	chromedriver!(No symbol) [0x7ff793f89f03]
+	chromedriver!GetHandleVerifier [0x7ff7944e58f9+329d89]
+	chromedriver!GetHandleVerifier [0x7ff7944dfe46+3242d6]
+	chromedriver!GetHandleVerifier [0x7ff7945030b2+347542]
+	chromedriver!GetHandleVerifier [0x7ff7941ed3d5+31865]
+	chromedriver!GetHandleVerifier [0x7ff7941f600c+3a49c]
+	chromedriver!GetHandleVerifier [0x7ff7941d9634+1dac4]
+	chromedriver!GetHandleVerifier [0x7ff7941d97e6+1dc76]
+	chromedriver!GetHandleVerifier [0x7ff7941be2f7+2787]
+	KERNEL32!BaseThreadInitThunk [0x7ffafb58e8d7+17]
+	ntdll!RtlUserThreadStart [0x7ffafbf4c3fc+2c]
+</t>
+  </si>
+  <si>
+    <t>N/A</t>
+  </si>
+  <si>
+    <t>FAIL</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> | Run: 2026-04-22 07:33</t>
+  </si>
+  <si>
+    <t>TC-RBAC-SES-04</t>
+  </si>
+  <si>
+    <t>Browser Back after logout</t>
+  </si>
+  <si>
+    <t>Protected page not accessible; redirect to /login</t>
+  </si>
+  <si>
+    <t>No active session</t>
+  </si>
+  <si>
+    <t>TC-RBAC-UI-04</t>
+  </si>
+  <si>
+    <t>Password field masking</t>
+  </si>
+  <si>
+    <t>GUI</t>
+  </si>
+  <si>
+    <t>Usability</t>
+  </si>
+  <si>
+    <t>Password characters shown as dots/asterisks</t>
+  </si>
+  <si>
+    <t>Password input type='password' (should be 'password')</t>
+  </si>
+  <si>
+    <t>N/A – UI-only check</t>
+  </si>
+  <si>
+    <t>TC-RBAC-AUTH-09</t>
+  </si>
+  <si>
+    <t>Forgot password – registered email</t>
+  </si>
+  <si>
+    <t>(none – forgot flow)</t>
+  </si>
+  <si>
+    <t>Confirmation message shown; reset email sent</t>
+  </si>
+  <si>
+    <t>Firebase sends reset email</t>
+  </si>
+  <si>
+    <t>Known bug: reset email not sent</t>
+  </si>
+  <si>
+    <t>TC-RBAC-AUTH-10</t>
+  </si>
+  <si>
+    <t>Forgot password – unregistered email</t>
+  </si>
+  <si>
+    <t>nobody@fake.com</t>
+  </si>
+  <si>
+    <t>Safe generic message (no email-exists leak)</t>
+  </si>
+  <si>
+    <t>No reset email sent</t>
+  </si>
+  <si>
+    <t>Known bug</t>
+  </si>
+  <si>
+    <t>TC-RBAC-AUTH-01</t>
+  </si>
+  <si>
+    <t>Register new account</t>
+  </si>
+  <si>
+    <t>newuser_TIMESTAMP@test.com</t>
+  </si>
+  <si>
+    <t>NewPass123!</t>
+  </si>
+  <si>
+    <t>Success message; redirect to dashboard</t>
+  </si>
+  <si>
+    <t>Firestore users/{uid} created; role='user'</t>
+  </si>
+  <si>
+    <t>Delete user via Firebase Admin SDK / Firestore</t>
+  </si>
+  <si>
+    <t>Known bug: conflicting UI message</t>
+  </si>
+  <si>
+    <t>F1 – RBAC Role &amp; Resource Access</t>
+  </si>
+  <si>
+    <t>selenium/scripts/test_rbac_roles.py</t>
+  </si>
+  <si>
+    <t>Role</t>
+  </si>
+  <si>
+    <t>URL / Action</t>
+  </si>
+  <si>
+    <t>Expected UI</t>
+  </si>
+  <si>
+    <t>Expected DB / Rule</t>
+  </si>
+  <si>
+    <t>Rollback</t>
+  </si>
+  <si>
+    <t>TC-RBAC-ROLE-02</t>
+  </si>
+  <si>
+    <t>User accesses learner dashboard</t>
+  </si>
+  <si>
+    <t>USER</t>
+  </si>
+  <si>
+    <t>/dashboard</t>
+  </si>
+  <si>
+    <t>Dashboard renders correctly; quiz cards visible</t>
+  </si>
+  <si>
+    <t>Firestore read allowed by security rules</t>
   </si>
   <si>
     <t>PENDING</t>
   </si>
   <si>
-    <t>TC-RBAC-NEG-01</t>
-  </si>
-  <si>
-    <t>Rapid repeated login clicks</t>
-  </si>
-  <si>
-    <t>Error Guessing</t>
-  </si>
-  <si>
-    <t>Negative</t>
-  </si>
-  <si>
-    <t>Single login action processed; no duplicate sessions</t>
-  </si>
-  <si>
-    <t>Only 1 auth token created</t>
-  </si>
-  <si>
-    <t>TC-RBAC-NEG-02</t>
-  </si>
-  <si>
-    <t>XSS payload in email field</t>
-  </si>
-  <si>
-    <t>Security</t>
-  </si>
-  <si>
-    <t>&lt;script&gt;alert('xss')&lt;/script&gt;</t>
-  </si>
-  <si>
-    <t>Input rejected; no script executed</t>
-  </si>
-  <si>
-    <t>No auth attempt or error logged</t>
-  </si>
-  <si>
-    <t>TC-RBAC-NEG-02b</t>
-  </si>
-  <si>
-    <t>SQL injection in password</t>
-  </si>
-  <si>
-    <t>' OR '1'='1; --</t>
-  </si>
-  <si>
-    <t>Login fails; no data exposure</t>
-  </si>
-  <si>
-    <t>TC-RBAC-AUTH-08</t>
-  </si>
-  <si>
-    <t>Google OAuth login</t>
-  </si>
-  <si>
-    <t>(Google account)</t>
-  </si>
-  <si>
-    <t>(OAuth flow)</t>
-  </si>
-  <si>
-    <t>Redirect to dashboard; profile synced</t>
-  </si>
-  <si>
-    <t>Firestore users/{uid} created with role='user'</t>
-  </si>
-  <si>
-    <t>Manual step: select Google account</t>
-  </si>
-  <si>
-    <t>TC-RBAC-ROLE-01</t>
-  </si>
-  <si>
-    <t>Guest access to protected route</t>
-  </si>
-  <si>
-    <t>Decision Table</t>
-  </si>
-  <si>
-    <t>(not logged in)</t>
-  </si>
-  <si>
-    <t>(none)</t>
-  </si>
-  <si>
-    <t>Redirect to /login page</t>
-  </si>
-  <si>
-    <t>Navigate to /profile while logged out</t>
-  </si>
-  <si>
-    <t>TC-RBAC-SES-03</t>
-  </si>
-  <si>
-    <t>Logout invalidates session</t>
-  </si>
-  <si>
-    <t>State Transition</t>
-  </si>
-  <si>
-    <t>Redirect to /login; protected pages blocked</t>
-  </si>
-  <si>
-    <t>Firebase ID token invalidated</t>
-  </si>
-  <si>
-    <t>N/A (logout is the action)</t>
-  </si>
-  <si>
-    <t>TC-RBAC-SES-04</t>
-  </si>
-  <si>
-    <t>Browser Back after logout</t>
-  </si>
-  <si>
-    <t>Protected page not accessible; redirect to /login</t>
-  </si>
-  <si>
-    <t>No active session</t>
-  </si>
-  <si>
-    <t>N/A</t>
-  </si>
-  <si>
-    <t>TC-RBAC-UI-04</t>
-  </si>
-  <si>
-    <t>Password field masking</t>
-  </si>
-  <si>
-    <t>GUI</t>
-  </si>
-  <si>
-    <t>Usability</t>
-  </si>
-  <si>
-    <t>Password characters shown as dots/asterisks</t>
-  </si>
-  <si>
-    <t>TC-RBAC-AUTH-09</t>
-  </si>
-  <si>
-    <t>Forgot password – registered email</t>
-  </si>
-  <si>
-    <t>(none – forgot flow)</t>
-  </si>
-  <si>
-    <t>Confirmation message shown; reset email sent</t>
-  </si>
-  <si>
-    <t>Firebase sends reset email</t>
-  </si>
-  <si>
-    <t>FAIL</t>
-  </si>
-  <si>
-    <t>Known bug: reset email not sent</t>
-  </si>
-  <si>
-    <t>TC-RBAC-AUTH-10</t>
-  </si>
-  <si>
-    <t>Forgot password – unregistered email</t>
-  </si>
-  <si>
-    <t>nobody@fake.com</t>
-  </si>
-  <si>
-    <t>Safe generic message (no email-exists leak)</t>
-  </si>
-  <si>
-    <t>No reset email sent</t>
-  </si>
-  <si>
-    <t>Known bug</t>
-  </si>
-  <si>
-    <t>TC-RBAC-AUTH-01</t>
-  </si>
-  <si>
-    <t>Register new account</t>
-  </si>
-  <si>
-    <t>newuser_TIMESTAMP@test.com</t>
-  </si>
-  <si>
-    <t>NewPass123!</t>
-  </si>
-  <si>
-    <t>Success message; redirect to dashboard</t>
-  </si>
-  <si>
-    <t>Firestore users/{uid} created; role='user'</t>
-  </si>
-  <si>
-    <t>Delete user via Firebase Admin SDK / Firestore</t>
-  </si>
-  <si>
-    <t>Known bug: conflicting UI message</t>
-  </si>
-  <si>
-    <t>F1 – RBAC Role &amp; Resource Access</t>
-  </si>
-  <si>
-    <t>selenium/scripts/test_rbac_roles.py</t>
-  </si>
-  <si>
-    <t>Role</t>
-  </si>
-  <si>
-    <t>URL / Action</t>
-  </si>
-  <si>
-    <t>Expected UI</t>
-  </si>
-  <si>
-    <t>Expected DB / Rule</t>
-  </si>
-  <si>
-    <t>Rollback</t>
-  </si>
-  <si>
-    <t>TC-RBAC-ROLE-02</t>
-  </si>
-  <si>
-    <t>User accesses learner dashboard</t>
-  </si>
-  <si>
-    <t>USER</t>
-  </si>
-  <si>
-    <t>/dashboard</t>
-  </si>
-  <si>
-    <t>Dashboard renders correctly; quiz cards visible</t>
-  </si>
-  <si>
-    <t>Firestore read allowed by security rules</t>
-  </si>
-  <si>
     <t>TC-RBAC-ROLE-03</t>
   </si>
   <si>
@@ -681,15 +765,6 @@
   </si>
   <si>
     <t>Firestore rule blocks read of non-public</t>
-  </si>
-  <si>
-    <t>nguyenvivi73@gmail.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  nguyenvivi73@gmail.com  </t>
-  </si>
-  <si>
-    <t xml:space="preserve">nguyenvivi73@gmail.com </t>
   </si>
 </sst>
 </file>
@@ -1397,7 +1472,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="10" spans="1:13" ht="38.25" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:13" ht="38.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A10" s="4" t="s">
         <v>46</v>
       </c>
@@ -1438,7 +1513,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="11" spans="1:13" ht="25.5" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:13" ht="25.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A11" s="6" t="s">
         <v>54</v>
       </c>
@@ -1477,7 +1552,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="12" spans="1:13" ht="25.5" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:13" ht="25.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A12" s="4" t="s">
         <v>62</v>
       </c>
@@ -1491,7 +1566,7 @@
         <v>56</v>
       </c>
       <c r="E12" t="s">
-        <v>220</v>
+        <v>64</v>
       </c>
       <c r="G12" s="4" t="s">
         <v>65</v>
@@ -1515,7 +1590,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="13" spans="1:13" ht="38.25" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:13" ht="38.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A13" s="6" t="s">
         <v>67</v>
       </c>
@@ -1556,7 +1631,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="14" spans="1:13" ht="38.25" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:13" ht="38.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A14" s="4" t="s">
         <v>73</v>
       </c>
@@ -1570,7 +1645,7 @@
         <v>56</v>
       </c>
       <c r="E14" t="s">
-        <v>220</v>
+        <v>64</v>
       </c>
       <c r="F14" s="4" t="s">
         <v>75</v>
@@ -1597,7 +1672,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="15" spans="1:13" ht="38.25" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:13" ht="38.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A15" s="6" t="s">
         <v>79</v>
       </c>
@@ -1611,54 +1686,54 @@
         <v>56</v>
       </c>
       <c r="E15" s="6" t="s">
-        <v>221</v>
+        <v>81</v>
       </c>
       <c r="F15" s="6" t="s">
         <v>57</v>
       </c>
       <c r="G15" s="6" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="H15" s="6" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="I15" s="6" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="J15" s="6" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="K15" s="6" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="L15" s="5" t="s">
         <v>34</v>
       </c>
       <c r="M15" s="6" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
     </row>
     <row r="16" spans="1:13" ht="127.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A16" s="4" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="E16" s="4" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="F16" s="4" t="s">
         <v>57</v>
       </c>
       <c r="G16" s="4" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="H16" s="4" t="s">
         <v>77</v>
@@ -1666,104 +1741,122 @@
       <c r="I16" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="J16" s="4"/>
-      <c r="K16" s="4"/>
+      <c r="J16" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="K16" s="4" t="s">
+        <v>95</v>
+      </c>
       <c r="L16" s="5" t="s">
-        <v>93</v>
-      </c>
-      <c r="M16" s="4"/>
+        <v>34</v>
+      </c>
+      <c r="M16" s="4" t="s">
+        <v>96</v>
+      </c>
     </row>
     <row r="17" spans="1:13" ht="25.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A17" s="6" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="E17" s="6" t="s">
-        <v>222</v>
+        <v>101</v>
       </c>
       <c r="F17" s="6" t="s">
         <v>57</v>
       </c>
       <c r="G17" s="6" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="H17" s="6" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="I17" s="6" t="s">
-        <v>83</v>
-      </c>
-      <c r="J17" s="6"/>
-      <c r="K17" s="6"/>
+        <v>84</v>
+      </c>
+      <c r="J17" s="6" t="s">
+        <v>104</v>
+      </c>
+      <c r="K17" s="6" t="s">
+        <v>105</v>
+      </c>
       <c r="L17" s="5" t="s">
-        <v>93</v>
-      </c>
-      <c r="M17" s="6"/>
-    </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.45">
+        <v>34</v>
+      </c>
+      <c r="M17" s="6" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="18" spans="1:13" ht="38.25" x14ac:dyDescent="0.45">
       <c r="A18" s="4" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>101</v>
+        <v>107</v>
       </c>
       <c r="C18" s="4" t="s">
         <v>38</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>102</v>
+        <v>108</v>
       </c>
       <c r="E18" s="4" t="s">
-        <v>103</v>
+        <v>109</v>
       </c>
       <c r="F18" s="4" t="s">
         <v>57</v>
       </c>
       <c r="G18" s="4" t="s">
-        <v>104</v>
+        <v>110</v>
       </c>
       <c r="H18" s="4" t="s">
-        <v>105</v>
+        <v>111</v>
       </c>
       <c r="I18" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="J18" s="4"/>
-      <c r="K18" s="4"/>
+      <c r="J18" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="K18" s="4" t="s">
+        <v>113</v>
+      </c>
       <c r="L18" s="5" t="s">
-        <v>93</v>
-      </c>
-      <c r="M18" s="4"/>
-    </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.45">
+        <v>34</v>
+      </c>
+      <c r="M18" s="4" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="19" spans="1:13" ht="51" x14ac:dyDescent="0.45">
       <c r="A19" s="6" t="s">
-        <v>106</v>
+        <v>115</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>107</v>
+        <v>116</v>
       </c>
       <c r="C19" s="6" t="s">
         <v>38</v>
       </c>
       <c r="D19" s="6" t="s">
-        <v>102</v>
+        <v>108</v>
       </c>
       <c r="E19" s="6" t="s">
-        <v>64</v>
+        <v>117</v>
       </c>
       <c r="F19" s="6" t="s">
-        <v>108</v>
+        <v>118</v>
       </c>
       <c r="G19" s="6" t="s">
-        <v>109</v>
+        <v>119</v>
       </c>
       <c r="H19" s="6" t="s">
         <v>77</v>
@@ -1771,19 +1864,25 @@
       <c r="I19" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="J19" s="6"/>
-      <c r="K19" s="6"/>
+      <c r="J19" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="K19" s="6" t="s">
+        <v>120</v>
+      </c>
       <c r="L19" s="5" t="s">
-        <v>93</v>
-      </c>
-      <c r="M19" s="6"/>
+        <v>34</v>
+      </c>
+      <c r="M19" s="6" t="s">
+        <v>114</v>
+      </c>
     </row>
     <row r="20" spans="1:13" ht="25.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A20" s="4" t="s">
-        <v>110</v>
+        <v>121</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>111</v>
+        <v>122</v>
       </c>
       <c r="C20" s="4" t="s">
         <v>25</v>
@@ -1792,50 +1891,54 @@
         <v>26</v>
       </c>
       <c r="E20" s="4" t="s">
-        <v>112</v>
+        <v>123</v>
       </c>
       <c r="F20" s="4" t="s">
-        <v>113</v>
+        <v>124</v>
       </c>
       <c r="G20" s="4" t="s">
-        <v>114</v>
+        <v>125</v>
       </c>
       <c r="H20" s="4" t="s">
-        <v>115</v>
+        <v>126</v>
       </c>
       <c r="I20" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="J20" s="4"/>
-      <c r="K20" s="4"/>
+      <c r="J20" s="4" t="s">
+        <v>127</v>
+      </c>
+      <c r="K20" s="4" t="s">
+        <v>128</v>
+      </c>
       <c r="L20" s="5" t="s">
-        <v>93</v>
+        <v>129</v>
       </c>
       <c r="M20" s="4" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.45">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="21" spans="1:13" ht="38.25" x14ac:dyDescent="0.45">
       <c r="A21" s="6" t="s">
-        <v>117</v>
+        <v>131</v>
       </c>
       <c r="B21" s="6" t="s">
-        <v>118</v>
+        <v>132</v>
       </c>
       <c r="C21" s="6" t="s">
-        <v>119</v>
+        <v>133</v>
       </c>
       <c r="D21" s="6" t="s">
-        <v>102</v>
+        <v>108</v>
       </c>
       <c r="E21" s="6" t="s">
-        <v>120</v>
+        <v>134</v>
       </c>
       <c r="F21" s="6" t="s">
-        <v>121</v>
+        <v>135</v>
       </c>
       <c r="G21" s="6" t="s">
-        <v>122</v>
+        <v>136</v>
       </c>
       <c r="H21" s="6" t="s">
         <v>77</v>
@@ -1843,126 +1946,148 @@
       <c r="I21" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="J21" s="6"/>
-      <c r="K21" s="6"/>
+      <c r="J21" s="6" t="s">
+        <v>137</v>
+      </c>
+      <c r="K21" s="6" t="s">
+        <v>138</v>
+      </c>
       <c r="L21" s="5" t="s">
-        <v>93</v>
+        <v>34</v>
       </c>
       <c r="M21" s="6" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.45">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="22" spans="1:13" ht="409.5" x14ac:dyDescent="0.45">
       <c r="A22" s="4" t="s">
-        <v>124</v>
+        <v>140</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>125</v>
+        <v>141</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>126</v>
+        <v>142</v>
       </c>
       <c r="D22" s="4" t="s">
         <v>26</v>
       </c>
       <c r="E22" s="4" t="s">
-        <v>64</v>
+        <v>117</v>
       </c>
       <c r="F22" s="4" t="s">
         <v>57</v>
       </c>
       <c r="G22" s="4" t="s">
-        <v>127</v>
+        <v>143</v>
       </c>
       <c r="H22" s="4" t="s">
-        <v>128</v>
+        <v>144</v>
       </c>
       <c r="I22" s="4" t="s">
-        <v>129</v>
-      </c>
-      <c r="J22" s="4"/>
-      <c r="K22" s="4"/>
+        <v>145</v>
+      </c>
+      <c r="J22" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="K22" s="4" t="s">
+        <v>147</v>
+      </c>
       <c r="L22" s="5" t="s">
-        <v>93</v>
-      </c>
-      <c r="M22" s="4"/>
-    </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.45">
+        <v>148</v>
+      </c>
+      <c r="M22" s="4" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="23" spans="1:13" ht="409.5" x14ac:dyDescent="0.45">
       <c r="A23" s="6" t="s">
-        <v>130</v>
+        <v>150</v>
       </c>
       <c r="B23" s="6" t="s">
-        <v>131</v>
+        <v>151</v>
       </c>
       <c r="C23" s="6" t="s">
-        <v>126</v>
+        <v>142</v>
       </c>
       <c r="D23" s="6" t="s">
-        <v>102</v>
+        <v>108</v>
       </c>
       <c r="E23" s="6" t="s">
-        <v>64</v>
+        <v>117</v>
       </c>
       <c r="F23" s="6" t="s">
         <v>57</v>
       </c>
       <c r="G23" s="6" t="s">
-        <v>132</v>
+        <v>152</v>
       </c>
       <c r="H23" s="6" t="s">
-        <v>133</v>
+        <v>153</v>
       </c>
       <c r="I23" s="6" t="s">
-        <v>134</v>
-      </c>
-      <c r="J23" s="6"/>
-      <c r="K23" s="6"/>
+        <v>147</v>
+      </c>
+      <c r="J23" s="6" t="s">
+        <v>146</v>
+      </c>
+      <c r="K23" s="6" t="s">
+        <v>147</v>
+      </c>
       <c r="L23" s="5" t="s">
-        <v>93</v>
-      </c>
-      <c r="M23" s="6"/>
-    </row>
-    <row r="24" spans="1:13" x14ac:dyDescent="0.45">
+        <v>148</v>
+      </c>
+      <c r="M23" s="6" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="24" spans="1:13" ht="25.5" x14ac:dyDescent="0.45">
       <c r="A24" s="4" t="s">
-        <v>135</v>
+        <v>154</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>136</v>
+        <v>155</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>137</v>
+        <v>156</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>138</v>
+        <v>157</v>
       </c>
       <c r="E24" s="4" t="s">
-        <v>64</v>
+        <v>117</v>
       </c>
       <c r="F24" s="4" t="s">
         <v>57</v>
       </c>
       <c r="G24" s="4" t="s">
-        <v>139</v>
+        <v>158</v>
       </c>
       <c r="H24" s="4" t="s">
-        <v>134</v>
+        <v>147</v>
       </c>
       <c r="I24" s="4" t="s">
-        <v>83</v>
-      </c>
-      <c r="J24" s="4"/>
-      <c r="K24" s="4"/>
+        <v>84</v>
+      </c>
+      <c r="J24" s="4" t="s">
+        <v>159</v>
+      </c>
+      <c r="K24" s="4" t="s">
+        <v>160</v>
+      </c>
       <c r="L24" s="5" t="s">
-        <v>93</v>
-      </c>
-      <c r="M24" s="4"/>
+        <v>34</v>
+      </c>
+      <c r="M24" s="4" t="s">
+        <v>149</v>
+      </c>
     </row>
     <row r="25" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A25" s="6" t="s">
-        <v>140</v>
+        <v>161</v>
       </c>
       <c r="B25" s="6" t="s">
-        <v>141</v>
+        <v>162</v>
       </c>
       <c r="C25" s="6" t="s">
         <v>25</v>
@@ -1971,16 +2096,16 @@
         <v>26</v>
       </c>
       <c r="E25" s="6" t="s">
-        <v>64</v>
+        <v>117</v>
       </c>
       <c r="F25" s="6" t="s">
-        <v>142</v>
+        <v>163</v>
       </c>
       <c r="G25" s="6" t="s">
-        <v>143</v>
+        <v>164</v>
       </c>
       <c r="H25" s="6" t="s">
-        <v>144</v>
+        <v>165</v>
       </c>
       <c r="I25" s="6" t="s">
         <v>51</v>
@@ -1988,18 +2113,18 @@
       <c r="J25" s="6"/>
       <c r="K25" s="6"/>
       <c r="L25" s="7" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="M25" s="6" t="s">
-        <v>146</v>
+        <v>166</v>
       </c>
     </row>
     <row r="26" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A26" s="4" t="s">
-        <v>147</v>
+        <v>167</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>148</v>
+        <v>168</v>
       </c>
       <c r="C26" s="4" t="s">
         <v>38</v>
@@ -2008,16 +2133,16 @@
         <v>26</v>
       </c>
       <c r="E26" s="4" t="s">
-        <v>149</v>
+        <v>169</v>
       </c>
       <c r="F26" s="4" t="s">
-        <v>121</v>
+        <v>135</v>
       </c>
       <c r="G26" s="4" t="s">
-        <v>150</v>
+        <v>170</v>
       </c>
       <c r="H26" s="4" t="s">
-        <v>151</v>
+        <v>171</v>
       </c>
       <c r="I26" s="4" t="s">
         <v>51</v>
@@ -2025,18 +2150,18 @@
       <c r="J26" s="4"/>
       <c r="K26" s="4"/>
       <c r="L26" s="7" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="M26" s="4" t="s">
-        <v>152</v>
+        <v>172</v>
       </c>
     </row>
     <row r="27" spans="1:13" ht="25.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A27" s="6" t="s">
-        <v>153</v>
+        <v>173</v>
       </c>
       <c r="B27" s="6" t="s">
-        <v>154</v>
+        <v>174</v>
       </c>
       <c r="C27" s="6" t="s">
         <v>25</v>
@@ -2045,27 +2170,27 @@
         <v>26</v>
       </c>
       <c r="E27" s="6" t="s">
-        <v>155</v>
+        <v>175</v>
       </c>
       <c r="F27" s="6" t="s">
-        <v>156</v>
+        <v>176</v>
       </c>
       <c r="G27" s="6" t="s">
-        <v>157</v>
+        <v>177</v>
       </c>
       <c r="H27" s="6" t="s">
-        <v>158</v>
+        <v>178</v>
       </c>
       <c r="I27" s="6" t="s">
-        <v>159</v>
+        <v>179</v>
       </c>
       <c r="J27" s="6"/>
       <c r="K27" s="6"/>
       <c r="L27" s="7" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="M27" s="6" t="s">
-        <v>160</v>
+        <v>180</v>
       </c>
     </row>
   </sheetData>
@@ -2079,8 +2204,8 @@
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="E8" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
-    <hyperlink ref="E10" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
-    <hyperlink ref="E14" r:id="rId3" xr:uid="{36C41BC0-033E-4BAD-8582-4CC29949F8E8}"/>
+    <hyperlink ref="E10" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
+    <hyperlink ref="E14" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2115,7 +2240,7 @@
         <v>2</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>161</v>
+        <v>181</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.45">
@@ -2131,7 +2256,7 @@
         <v>6</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>162</v>
+        <v>182</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.45">
@@ -2142,19 +2267,19 @@
         <v>11</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>163</v>
+        <v>183</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>164</v>
+        <v>184</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>165</v>
+        <v>185</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>166</v>
+        <v>186</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>167</v>
+        <v>187</v>
       </c>
       <c r="H5" s="3" t="s">
         <v>21</v>
@@ -2165,271 +2290,271 @@
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A6" s="4" t="s">
-        <v>168</v>
+        <v>188</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>169</v>
+        <v>189</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>170</v>
+        <v>190</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>171</v>
+        <v>191</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>172</v>
+        <v>192</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>173</v>
+        <v>193</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>134</v>
+        <v>147</v>
       </c>
       <c r="H6" s="5" t="s">
-        <v>93</v>
+        <v>194</v>
       </c>
       <c r="I6" s="4"/>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A7" s="6" t="s">
-        <v>174</v>
+        <v>195</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>175</v>
+        <v>196</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>170</v>
+        <v>190</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>176</v>
+        <v>197</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>177</v>
+        <v>198</v>
       </c>
       <c r="F7" s="6" t="s">
-        <v>178</v>
+        <v>199</v>
       </c>
       <c r="G7" s="6" t="s">
-        <v>134</v>
+        <v>147</v>
       </c>
       <c r="H7" s="5" t="s">
-        <v>93</v>
+        <v>194</v>
       </c>
       <c r="I7" s="6"/>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A8" s="4" t="s">
-        <v>179</v>
+        <v>200</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>180</v>
+        <v>201</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>170</v>
+        <v>190</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>181</v>
+        <v>202</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>182</v>
+        <v>203</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>183</v>
+        <v>204</v>
       </c>
       <c r="G8" s="4" t="s">
-        <v>134</v>
+        <v>147</v>
       </c>
       <c r="H8" s="5" t="s">
-        <v>93</v>
+        <v>194</v>
       </c>
       <c r="I8" s="4"/>
     </row>
     <row r="9" spans="1:9" ht="25.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A9" s="6" t="s">
-        <v>184</v>
+        <v>205</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>185</v>
+        <v>206</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>186</v>
+        <v>207</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>187</v>
+        <v>208</v>
       </c>
       <c r="E9" s="6" t="s">
-        <v>188</v>
+        <v>209</v>
       </c>
       <c r="F9" s="6" t="s">
-        <v>189</v>
+        <v>210</v>
       </c>
       <c r="G9" s="6" t="s">
-        <v>134</v>
+        <v>147</v>
       </c>
       <c r="H9" s="5" t="s">
-        <v>93</v>
+        <v>194</v>
       </c>
       <c r="I9" s="6"/>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A10" s="4" t="s">
-        <v>190</v>
+        <v>211</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>191</v>
+        <v>212</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>186</v>
+        <v>207</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>192</v>
+        <v>213</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>193</v>
+        <v>214</v>
       </c>
       <c r="F10" s="4" t="s">
+        <v>215</v>
+      </c>
+      <c r="G10" s="4" t="s">
+        <v>147</v>
+      </c>
+      <c r="H10" s="5" t="s">
         <v>194</v>
-      </c>
-      <c r="G10" s="4" t="s">
-        <v>134</v>
-      </c>
-      <c r="H10" s="5" t="s">
-        <v>93</v>
       </c>
       <c r="I10" s="4"/>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A11" s="6" t="s">
-        <v>195</v>
+        <v>216</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>196</v>
+        <v>217</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>197</v>
+        <v>218</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>192</v>
+        <v>213</v>
       </c>
       <c r="E11" s="6" t="s">
-        <v>198</v>
+        <v>219</v>
       </c>
       <c r="F11" s="6" t="s">
-        <v>199</v>
+        <v>220</v>
       </c>
       <c r="G11" s="6" t="s">
-        <v>134</v>
+        <v>147</v>
       </c>
       <c r="H11" s="5" t="s">
-        <v>93</v>
+        <v>194</v>
       </c>
       <c r="I11" s="6"/>
     </row>
     <row r="12" spans="1:9" ht="25.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A12" s="4" t="s">
-        <v>200</v>
+        <v>221</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>201</v>
+        <v>222</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>170</v>
+        <v>190</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>202</v>
+        <v>223</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>203</v>
+        <v>224</v>
       </c>
       <c r="F12" s="4" t="s">
-        <v>204</v>
+        <v>225</v>
       </c>
       <c r="G12" s="4" t="s">
-        <v>134</v>
+        <v>147</v>
       </c>
       <c r="H12" s="5" t="s">
-        <v>93</v>
+        <v>194</v>
       </c>
       <c r="I12" s="4"/>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A13" s="6" t="s">
-        <v>205</v>
+        <v>226</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>206</v>
+        <v>227</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>170</v>
+        <v>190</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>207</v>
+        <v>228</v>
       </c>
       <c r="E13" s="6" t="s">
-        <v>208</v>
+        <v>229</v>
       </c>
       <c r="F13" s="6" t="s">
-        <v>209</v>
+        <v>230</v>
       </c>
       <c r="G13" s="6" t="s">
-        <v>134</v>
+        <v>147</v>
       </c>
       <c r="H13" s="5" t="s">
-        <v>93</v>
+        <v>194</v>
       </c>
       <c r="I13" s="6"/>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A14" s="4" t="s">
-        <v>210</v>
+        <v>231</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>211</v>
+        <v>232</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>186</v>
+        <v>207</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>212</v>
+        <v>233</v>
       </c>
       <c r="E14" s="4" t="s">
-        <v>213</v>
+        <v>234</v>
       </c>
       <c r="F14" s="4" t="s">
-        <v>214</v>
+        <v>235</v>
       </c>
       <c r="G14" s="4" t="s">
-        <v>134</v>
+        <v>147</v>
       </c>
       <c r="H14" s="5" t="s">
-        <v>93</v>
+        <v>194</v>
       </c>
       <c r="I14" s="4"/>
     </row>
     <row r="15" spans="1:9" ht="25.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A15" s="6" t="s">
-        <v>215</v>
+        <v>236</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>216</v>
+        <v>237</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>170</v>
+        <v>190</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>217</v>
+        <v>238</v>
       </c>
       <c r="E15" s="6" t="s">
-        <v>218</v>
+        <v>239</v>
       </c>
       <c r="F15" s="6" t="s">
-        <v>219</v>
+        <v>240</v>
       </c>
       <c r="G15" s="6" t="s">
-        <v>134</v>
+        <v>147</v>
       </c>
       <c r="H15" s="5" t="s">
-        <v>93</v>
+        <v>194</v>
       </c>
       <c r="I15" s="6"/>
     </row>

</xml_diff>

<commit_message>
feat: add login test automation suite with Excel-driven test cases
</commit_message>
<xml_diff>
--- a/data/TC_Login.xlsx
+++ b/data/TC_Login.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Đồ án\quiz-trivia-tooltest\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{75D4A7CB-7469-4128-8DAD-A83211579780}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95BB8726-C39B-4C8A-B59A-449F40EB7767}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="34452" yWindow="1188" windowWidth="30936" windowHeight="16776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="372" uniqueCount="241">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="372" uniqueCount="245">
   <si>
     <t>Project</t>
   </si>
@@ -461,85 +461,76 @@
     <t>N/A (logout is the action)</t>
   </si>
   <si>
-    <t xml:space="preserve">Logout UI interaction failed: Message: 
-Stacktrace:
-	chromedriver!GetHandleVerifier [0x7ff7941d0245+146d5]
-	chromedriver!GetHandleVerifier [0x7ff7941d02b0+14740]
-	chromedriver!(No symbol) [0x7ff793f3d7cd]
-	chromedriver!(No symbol) [0x7ff793f96c4e]
-	chromedriver!(No symbol) [0x7ff793f96f5c]
-	chromedriver!(No symbol) [0x7ff793fe7cc7]
-	chromedriver!(No symbol) [0x7ff793fe4818]
-	chromedriver!(No symbol) [0x7ff793f89018]
-	chromedriver!(No symbol) [0x7ff793f89f03]
-	chromedriver!GetHandleVerifier [0x7ff7944e58f9+329d89]
-	chromedriver!GetHandleVerifier [0x7ff7944dfe46+3242d6]
-	chromedriver!GetHandleVerifier [0x7ff7945030b2+347542]
-	chromedriver!GetHandleVerifier [0x7ff7941ed3d5+31865]
-	chromedriver!GetHandleVerifier [0x7ff7941f600c+3a49c]
-	chromedriver!GetHandleVerifier [0x7ff7941d9634+1dac4]
-	chromedriver!GetHandleVerifier [0x7ff7941d97e6+1dc76]
-	chromedriver!GetHandleVerifier [0x7ff7941be2f7+2787]
-	KERNEL32!BaseThreadInitThunk [0x7ffafb58e8d7+17]
-	ntdll!RtlUserThreadStart [0x7ffafbf4c3fc+2c]
-</t>
+    <t>After logout → https://datn-quizapp.web.app/login; Redirect to /login: True; /dashboard blocked: True</t>
+  </si>
+  <si>
+    <t>Firebase ID token invalidated (Firebase client SDK revokes local token on signOut)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> | Run: 2026-04-22 07:33 | Run: 2026-04-22 09:13</t>
+  </si>
+  <si>
+    <t>TC-RBAC-SES-04</t>
+  </si>
+  <si>
+    <t>Browser Back after logout</t>
+  </si>
+  <si>
+    <t>Protected page not accessible; redirect to /login</t>
+  </si>
+  <si>
+    <t>No active session</t>
   </si>
   <si>
     <t>N/A</t>
   </si>
   <si>
+    <t>After Back → https://datn-quizapp.web.app/login; Protected page inaccessible: True</t>
+  </si>
+  <si>
+    <t>No active session (back-navigation does not restore Firebase token)</t>
+  </si>
+  <si>
+    <t>TC-RBAC-UI-04</t>
+  </si>
+  <si>
+    <t>Password field masking</t>
+  </si>
+  <si>
+    <t>GUI</t>
+  </si>
+  <si>
+    <t>Usability</t>
+  </si>
+  <si>
+    <t>Password characters shown as dots/asterisks</t>
+  </si>
+  <si>
+    <t>Password input type='password' (should be 'password')</t>
+  </si>
+  <si>
+    <t>N/A – UI-only check</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> | Run: 2026-04-22 07:33</t>
+  </si>
+  <si>
+    <t>TC-RBAC-AUTH-09</t>
+  </si>
+  <si>
+    <t>Forgot password – registered email</t>
+  </si>
+  <si>
+    <t>(none – forgot flow)</t>
+  </si>
+  <si>
+    <t>Confirmation message shown; reset email sent</t>
+  </si>
+  <si>
+    <t>Firebase sends reset email</t>
+  </si>
+  <si>
     <t>FAIL</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> | Run: 2026-04-22 07:33</t>
-  </si>
-  <si>
-    <t>TC-RBAC-SES-04</t>
-  </si>
-  <si>
-    <t>Browser Back after logout</t>
-  </si>
-  <si>
-    <t>Protected page not accessible; redirect to /login</t>
-  </si>
-  <si>
-    <t>No active session</t>
-  </si>
-  <si>
-    <t>TC-RBAC-UI-04</t>
-  </si>
-  <si>
-    <t>Password field masking</t>
-  </si>
-  <si>
-    <t>GUI</t>
-  </si>
-  <si>
-    <t>Usability</t>
-  </si>
-  <si>
-    <t>Password characters shown as dots/asterisks</t>
-  </si>
-  <si>
-    <t>Password input type='password' (should be 'password')</t>
-  </si>
-  <si>
-    <t>N/A – UI-only check</t>
-  </si>
-  <si>
-    <t>TC-RBAC-AUTH-09</t>
-  </si>
-  <si>
-    <t>Forgot password – registered email</t>
-  </si>
-  <si>
-    <t>(none – forgot flow)</t>
-  </si>
-  <si>
-    <t>Confirmation message shown; reset email sent</t>
-  </si>
-  <si>
-    <t>Firebase sends reset email</t>
   </si>
   <si>
     <t>Known bug: reset email not sent</t>
@@ -1795,7 +1786,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="18" spans="1:13" ht="38.25" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:13" ht="38.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A18" s="4" t="s">
         <v>106</v>
       </c>
@@ -1836,7 +1827,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="19" spans="1:13" ht="51" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:13" ht="51" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A19" s="6" t="s">
         <v>115</v>
       </c>
@@ -1918,7 +1909,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="21" spans="1:13" ht="38.25" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:13" ht="38.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A21" s="6" t="s">
         <v>131</v>
       </c>
@@ -1959,7 +1950,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="22" spans="1:13" ht="409.5" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:13" ht="409.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A22" s="4" t="s">
         <v>140</v>
       </c>
@@ -1994,18 +1985,18 @@
         <v>147</v>
       </c>
       <c r="L22" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="M22" s="4" t="s">
         <v>148</v>
       </c>
-      <c r="M22" s="4" t="s">
+    </row>
+    <row r="23" spans="1:13" ht="409.5" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A23" s="6" t="s">
         <v>149</v>
       </c>
-    </row>
-    <row r="23" spans="1:13" ht="409.5" x14ac:dyDescent="0.45">
-      <c r="A23" s="6" t="s">
+      <c r="B23" s="6" t="s">
         <v>150</v>
-      </c>
-      <c r="B23" s="6" t="s">
-        <v>151</v>
       </c>
       <c r="C23" s="6" t="s">
         <v>142</v>
@@ -2020,39 +2011,39 @@
         <v>57</v>
       </c>
       <c r="G23" s="6" t="s">
+        <v>151</v>
+      </c>
+      <c r="H23" s="6" t="s">
         <v>152</v>
       </c>
-      <c r="H23" s="6" t="s">
+      <c r="I23" s="6" t="s">
         <v>153</v>
       </c>
-      <c r="I23" s="6" t="s">
-        <v>147</v>
-      </c>
       <c r="J23" s="6" t="s">
-        <v>146</v>
+        <v>154</v>
       </c>
       <c r="K23" s="6" t="s">
-        <v>147</v>
+        <v>155</v>
       </c>
       <c r="L23" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="M23" s="6" t="s">
         <v>148</v>
       </c>
-      <c r="M23" s="6" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="24" spans="1:13" ht="25.5" x14ac:dyDescent="0.45">
+    </row>
+    <row r="24" spans="1:13" ht="25.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A24" s="4" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="E24" s="4" t="s">
         <v>117</v>
@@ -2061,33 +2052,33 @@
         <v>57</v>
       </c>
       <c r="G24" s="4" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="H24" s="4" t="s">
-        <v>147</v>
+        <v>153</v>
       </c>
       <c r="I24" s="4" t="s">
         <v>84</v>
       </c>
       <c r="J24" s="4" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="K24" s="4" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="L24" s="5" t="s">
         <v>34</v>
       </c>
       <c r="M24" s="4" t="s">
-        <v>149</v>
+        <v>163</v>
       </c>
     </row>
     <row r="25" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A25" s="6" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="B25" s="6" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="C25" s="6" t="s">
         <v>25</v>
@@ -2099,13 +2090,13 @@
         <v>117</v>
       </c>
       <c r="F25" s="6" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="G25" s="6" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="H25" s="6" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="I25" s="6" t="s">
         <v>51</v>
@@ -2113,18 +2104,18 @@
       <c r="J25" s="6"/>
       <c r="K25" s="6"/>
       <c r="L25" s="7" t="s">
-        <v>148</v>
+        <v>169</v>
       </c>
       <c r="M25" s="6" t="s">
-        <v>166</v>
+        <v>170</v>
       </c>
     </row>
     <row r="26" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A26" s="4" t="s">
-        <v>167</v>
+        <v>171</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>168</v>
+        <v>172</v>
       </c>
       <c r="C26" s="4" t="s">
         <v>38</v>
@@ -2133,16 +2124,16 @@
         <v>26</v>
       </c>
       <c r="E26" s="4" t="s">
-        <v>169</v>
+        <v>173</v>
       </c>
       <c r="F26" s="4" t="s">
         <v>135</v>
       </c>
       <c r="G26" s="4" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
       <c r="H26" s="4" t="s">
-        <v>171</v>
+        <v>175</v>
       </c>
       <c r="I26" s="4" t="s">
         <v>51</v>
@@ -2150,18 +2141,18 @@
       <c r="J26" s="4"/>
       <c r="K26" s="4"/>
       <c r="L26" s="7" t="s">
-        <v>148</v>
+        <v>169</v>
       </c>
       <c r="M26" s="4" t="s">
-        <v>172</v>
+        <v>176</v>
       </c>
     </row>
     <row r="27" spans="1:13" ht="25.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A27" s="6" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
       <c r="B27" s="6" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="C27" s="6" t="s">
         <v>25</v>
@@ -2170,27 +2161,27 @@
         <v>26</v>
       </c>
       <c r="E27" s="6" t="s">
-        <v>175</v>
+        <v>179</v>
       </c>
       <c r="F27" s="6" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="G27" s="6" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="H27" s="6" t="s">
-        <v>178</v>
+        <v>182</v>
       </c>
       <c r="I27" s="6" t="s">
-        <v>179</v>
+        <v>183</v>
       </c>
       <c r="J27" s="6"/>
       <c r="K27" s="6"/>
       <c r="L27" s="7" t="s">
-        <v>148</v>
+        <v>169</v>
       </c>
       <c r="M27" s="6" t="s">
-        <v>180</v>
+        <v>184</v>
       </c>
     </row>
   </sheetData>
@@ -2240,7 +2231,7 @@
         <v>2</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>181</v>
+        <v>185</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.45">
@@ -2256,7 +2247,7 @@
         <v>6</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>182</v>
+        <v>186</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.45">
@@ -2267,19 +2258,19 @@
         <v>11</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>183</v>
+        <v>187</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>184</v>
+        <v>188</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>185</v>
+        <v>189</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>186</v>
+        <v>190</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>187</v>
+        <v>191</v>
       </c>
       <c r="H5" s="3" t="s">
         <v>21</v>
@@ -2290,271 +2281,271 @@
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A6" s="4" t="s">
-        <v>188</v>
+        <v>192</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>189</v>
+        <v>193</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>190</v>
+        <v>194</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>191</v>
+        <v>195</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>192</v>
+        <v>196</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>193</v>
+        <v>197</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>147</v>
+        <v>153</v>
       </c>
       <c r="H6" s="5" t="s">
-        <v>194</v>
+        <v>198</v>
       </c>
       <c r="I6" s="4"/>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A7" s="6" t="s">
-        <v>195</v>
+        <v>199</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>196</v>
+        <v>200</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>190</v>
+        <v>194</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>197</v>
+        <v>201</v>
       </c>
       <c r="E7" s="6" t="s">
+        <v>202</v>
+      </c>
+      <c r="F7" s="6" t="s">
+        <v>203</v>
+      </c>
+      <c r="G7" s="6" t="s">
+        <v>153</v>
+      </c>
+      <c r="H7" s="5" t="s">
         <v>198</v>
-      </c>
-      <c r="F7" s="6" t="s">
-        <v>199</v>
-      </c>
-      <c r="G7" s="6" t="s">
-        <v>147</v>
-      </c>
-      <c r="H7" s="5" t="s">
-        <v>194</v>
       </c>
       <c r="I7" s="6"/>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A8" s="4" t="s">
-        <v>200</v>
+        <v>204</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>201</v>
+        <v>205</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>190</v>
+        <v>194</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>202</v>
+        <v>206</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>203</v>
+        <v>207</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>204</v>
+        <v>208</v>
       </c>
       <c r="G8" s="4" t="s">
-        <v>147</v>
+        <v>153</v>
       </c>
       <c r="H8" s="5" t="s">
-        <v>194</v>
+        <v>198</v>
       </c>
       <c r="I8" s="4"/>
     </row>
     <row r="9" spans="1:9" ht="25.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A9" s="6" t="s">
-        <v>205</v>
+        <v>209</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>206</v>
+        <v>210</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>207</v>
+        <v>211</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>208</v>
+        <v>212</v>
       </c>
       <c r="E9" s="6" t="s">
-        <v>209</v>
+        <v>213</v>
       </c>
       <c r="F9" s="6" t="s">
-        <v>210</v>
+        <v>214</v>
       </c>
       <c r="G9" s="6" t="s">
-        <v>147</v>
+        <v>153</v>
       </c>
       <c r="H9" s="5" t="s">
-        <v>194</v>
+        <v>198</v>
       </c>
       <c r="I9" s="6"/>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A10" s="4" t="s">
+        <v>215</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>216</v>
+      </c>
+      <c r="C10" s="4" t="s">
         <v>211</v>
       </c>
-      <c r="B10" s="4" t="s">
-        <v>212</v>
-      </c>
-      <c r="C10" s="4" t="s">
-        <v>207</v>
-      </c>
       <c r="D10" s="4" t="s">
-        <v>213</v>
+        <v>217</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>214</v>
+        <v>218</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>215</v>
+        <v>219</v>
       </c>
       <c r="G10" s="4" t="s">
-        <v>147</v>
+        <v>153</v>
       </c>
       <c r="H10" s="5" t="s">
-        <v>194</v>
+        <v>198</v>
       </c>
       <c r="I10" s="4"/>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A11" s="6" t="s">
-        <v>216</v>
+        <v>220</v>
       </c>
       <c r="B11" s="6" t="s">
+        <v>221</v>
+      </c>
+      <c r="C11" s="6" t="s">
+        <v>222</v>
+      </c>
+      <c r="D11" s="6" t="s">
         <v>217</v>
       </c>
-      <c r="C11" s="6" t="s">
-        <v>218</v>
-      </c>
-      <c r="D11" s="6" t="s">
-        <v>213</v>
-      </c>
       <c r="E11" s="6" t="s">
-        <v>219</v>
+        <v>223</v>
       </c>
       <c r="F11" s="6" t="s">
-        <v>220</v>
+        <v>224</v>
       </c>
       <c r="G11" s="6" t="s">
-        <v>147</v>
+        <v>153</v>
       </c>
       <c r="H11" s="5" t="s">
-        <v>194</v>
+        <v>198</v>
       </c>
       <c r="I11" s="6"/>
     </row>
     <row r="12" spans="1:9" ht="25.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A12" s="4" t="s">
-        <v>221</v>
+        <v>225</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>190</v>
+        <v>194</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>223</v>
+        <v>227</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>224</v>
+        <v>228</v>
       </c>
       <c r="F12" s="4" t="s">
-        <v>225</v>
+        <v>229</v>
       </c>
       <c r="G12" s="4" t="s">
-        <v>147</v>
+        <v>153</v>
       </c>
       <c r="H12" s="5" t="s">
-        <v>194</v>
+        <v>198</v>
       </c>
       <c r="I12" s="4"/>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A13" s="6" t="s">
-        <v>226</v>
+        <v>230</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>227</v>
+        <v>231</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>190</v>
+        <v>194</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>228</v>
+        <v>232</v>
       </c>
       <c r="E13" s="6" t="s">
-        <v>229</v>
+        <v>233</v>
       </c>
       <c r="F13" s="6" t="s">
-        <v>230</v>
+        <v>234</v>
       </c>
       <c r="G13" s="6" t="s">
-        <v>147</v>
+        <v>153</v>
       </c>
       <c r="H13" s="5" t="s">
-        <v>194</v>
+        <v>198</v>
       </c>
       <c r="I13" s="6"/>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A14" s="4" t="s">
-        <v>231</v>
+        <v>235</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>207</v>
+        <v>211</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>233</v>
+        <v>237</v>
       </c>
       <c r="E14" s="4" t="s">
-        <v>234</v>
+        <v>238</v>
       </c>
       <c r="F14" s="4" t="s">
-        <v>235</v>
+        <v>239</v>
       </c>
       <c r="G14" s="4" t="s">
-        <v>147</v>
+        <v>153</v>
       </c>
       <c r="H14" s="5" t="s">
-        <v>194</v>
+        <v>198</v>
       </c>
       <c r="I14" s="4"/>
     </row>
     <row r="15" spans="1:9" ht="25.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A15" s="6" t="s">
-        <v>236</v>
+        <v>240</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>237</v>
+        <v>241</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>190</v>
+        <v>194</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>238</v>
+        <v>242</v>
       </c>
       <c r="E15" s="6" t="s">
-        <v>239</v>
+        <v>243</v>
       </c>
       <c r="F15" s="6" t="s">
-        <v>240</v>
+        <v>244</v>
       </c>
       <c r="G15" s="6" t="s">
-        <v>147</v>
+        <v>153</v>
       </c>
       <c r="H15" s="5" t="s">
-        <v>194</v>
+        <v>198</v>
       </c>
       <c r="I15" s="6"/>
     </row>

</xml_diff>